<commit_message>
add: Correcion pdf retenciones, y totalizacion en la cabecera de retencion.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/Servicios.xlsx
+++ b/api/src/main/resources/importaciones/Servicios.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1399244-22F4-4FD2-8818-563A0B2CA0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B14CA8-4144-4ED2-997D-B0324A92AD9C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,9 +239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,9 +279,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -314,9 +314,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -349,9 +366,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -525,8 +559,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.42578125" customWidth="1"/>
     <col min="4" max="4" width="20" style="1" customWidth="1"/>
@@ -750,43 +784,16 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8" t="s">
-        <v>7</v>
-      </c>
-      <c r="H8" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" t="s">
-        <v>48</v>
-      </c>
-      <c r="K8" t="s">
-        <v>51</v>
-      </c>
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="D8"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
@@ -804,21 +811,21 @@
         <v>44</v>
       </c>
       <c r="I9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J9" t="s">
         <v>48</v>
       </c>
       <c r="K9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
@@ -842,15 +849,15 @@
         <v>48</v>
       </c>
       <c r="K10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
@@ -868,21 +875,21 @@
         <v>44</v>
       </c>
       <c r="I11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J11" t="s">
         <v>48</v>
       </c>
       <c r="K11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
@@ -900,21 +907,21 @@
         <v>44</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J12" t="s">
         <v>48</v>
       </c>
       <c r="K12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
@@ -932,21 +939,21 @@
         <v>44</v>
       </c>
       <c r="I13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J13" t="s">
         <v>48</v>
       </c>
       <c r="K13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
@@ -964,21 +971,21 @@
         <v>44</v>
       </c>
       <c r="I14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
       </c>
       <c r="K14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
@@ -996,21 +1003,21 @@
         <v>44</v>
       </c>
       <c r="I15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J15" t="s">
         <v>48</v>
       </c>
       <c r="K15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
@@ -1034,15 +1041,15 @@
         <v>48</v>
       </c>
       <c r="K16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
@@ -1060,21 +1067,21 @@
         <v>44</v>
       </c>
       <c r="I17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J17" t="s">
         <v>48</v>
       </c>
       <c r="K17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
         <v>8</v>
@@ -1092,21 +1099,21 @@
         <v>44</v>
       </c>
       <c r="I18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J18" t="s">
         <v>48</v>
       </c>
       <c r="K18" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
@@ -1124,21 +1131,21 @@
         <v>44</v>
       </c>
       <c r="I19" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J19" t="s">
         <v>48</v>
       </c>
       <c r="K19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
@@ -1156,44 +1163,76 @@
         <v>44</v>
       </c>
       <c r="I20" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J20" t="s">
         <v>48</v>
       </c>
       <c r="K20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21" t="s">
+        <v>7</v>
+      </c>
+      <c r="H21" t="s">
+        <v>44</v>
+      </c>
+      <c r="I21" t="s">
+        <v>47</v>
+      </c>
+      <c r="J21" t="s">
+        <v>48</v>
+      </c>
+      <c r="K21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21">
-        <v>2</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
-      <c r="F21" t="s">
-        <v>7</v>
-      </c>
-      <c r="H21" t="s">
-        <v>44</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22" t="s">
+        <v>7</v>
+      </c>
+      <c r="H22" t="s">
+        <v>44</v>
+      </c>
+      <c r="I22" t="s">
         <v>46</v>
       </c>
-      <c r="J21" t="s">
-        <v>48</v>
-      </c>
-      <c r="K21" t="s">
+      <c r="J22" t="s">
+        <v>48</v>
+      </c>
+      <c r="K22" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1207,7 +1246,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -1217,7 +1256,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>

</xml_diff>